<commit_message>
Step 10 working clock and countdown
</commit_message>
<xml_diff>
--- a/sync/prayer_db.xlsx
+++ b/sync/prayer_db.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/arman/Desktop/Waqt_App/sync/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{62D50C7E-B335-584C-B747-C61CFED2BBCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC9B485-B389-8B42-BEC6-3440F93063D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{8B6FC42C-4124-1A45-A3FA-D13FD9B78F6A}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15600" xr2:uid="{8B6FC42C-4124-1A45-A3FA-D13FD9B78F6A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="31">
   <si>
     <t>Date</t>
   </si>
@@ -105,6 +105,33 @@
   </si>
   <si>
     <t>21:37</t>
+  </si>
+  <si>
+    <t>Fajr_Iqamah</t>
+  </si>
+  <si>
+    <t>05:45</t>
+  </si>
+  <si>
+    <t>Dhuhr_Iqamah</t>
+  </si>
+  <si>
+    <t>Asr_Iqamah</t>
+  </si>
+  <si>
+    <t>Maghrib_Iqamah</t>
+  </si>
+  <si>
+    <t>Isha_Iqamah</t>
+  </si>
+  <si>
+    <t>14:00</t>
+  </si>
+  <si>
+    <t>17:00</t>
+  </si>
+  <si>
+    <t>22:00</t>
   </si>
 </sst>
 </file>
@@ -477,30 +504,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D9F3147-B029-C84B-A6D4-128D9068F6DF}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="16384" width="10.83203125" style="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="K1" s="1" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -508,19 +553,34 @@
         <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="G2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="I2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="K2" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -528,19 +588,34 @@
         <v>10</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="G3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="I3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="K3" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -548,16 +623,31 @@
         <v>11</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="G4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="I4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>21</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
If new year loaded, deletes old year too
</commit_message>
<xml_diff>
--- a/sync/prayer_db.xlsx
+++ b/sync/prayer_db.xlsx
@@ -842,7 +842,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>14:39</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -889,7 +889,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -1124,7 +1124,7 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>14:46</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -1171,7 +1171,7 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>14:46</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -1641,7 +1641,7 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>14:57</t>
+          <t>14:58</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -1688,7 +1688,7 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>14:58</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -2017,7 +2017,7 @@
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:08</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -2534,7 +2534,7 @@
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:19</t>
         </is>
       </c>
       <c r="I45" t="inlineStr"/>
@@ -2581,7 +2581,7 @@
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="I46" t="inlineStr"/>
@@ -2628,7 +2628,7 @@
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>15:21</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -2675,7 +2675,7 @@
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>15:21</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="I48" t="inlineStr"/>
@@ -2722,7 +2722,7 @@
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
@@ -2816,7 +2816,7 @@
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
@@ -2863,7 +2863,7 @@
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -2910,7 +2910,7 @@
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="I53" t="inlineStr"/>
@@ -2957,7 +2957,7 @@
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="I54" t="inlineStr"/>
@@ -3004,7 +3004,7 @@
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:29</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -3427,7 +3427,7 @@
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>15:36</t>
+          <t>15:37</t>
         </is>
       </c>
       <c r="I64" t="inlineStr"/>
@@ -3662,7 +3662,7 @@
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -4179,7 +4179,7 @@
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>16:48</t>
+          <t>16:49</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -4649,7 +4649,7 @@
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>16:54</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="I90" t="inlineStr"/>
@@ -5307,7 +5307,7 @@
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:02</t>
         </is>
       </c>
       <c r="I104" t="inlineStr"/>
@@ -6341,7 +6341,7 @@
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="I126" t="inlineStr"/>
@@ -6717,7 +6717,7 @@
       <c r="G134" t="inlineStr"/>
       <c r="H134" t="inlineStr">
         <is>
-          <t>17:13</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="I134" t="inlineStr"/>
@@ -7516,7 +7516,7 @@
       <c r="G151" t="inlineStr"/>
       <c r="H151" t="inlineStr">
         <is>
-          <t>17:19</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="I151" t="inlineStr"/>
@@ -7657,7 +7657,7 @@
       <c r="G154" t="inlineStr"/>
       <c r="H154" t="inlineStr">
         <is>
-          <t>17:20</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="I154" t="inlineStr"/>
@@ -7798,7 +7798,7 @@
       <c r="G157" t="inlineStr"/>
       <c r="H157" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="I157" t="inlineStr"/>
@@ -10007,7 +10007,7 @@
       <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr">
         <is>
-          <t>17:27</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="I204" t="inlineStr"/>
@@ -10712,7 +10712,7 @@
       <c r="G219" t="inlineStr"/>
       <c r="H219" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="I219" t="inlineStr"/>
@@ -10947,7 +10947,7 @@
       <c r="G224" t="inlineStr"/>
       <c r="H224" t="inlineStr">
         <is>
-          <t>17:18</t>
+          <t>17:17</t>
         </is>
       </c>
       <c r="I224" t="inlineStr"/>
@@ -11746,7 +11746,7 @@
       <c r="G241" t="inlineStr"/>
       <c r="H241" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="I241" t="inlineStr"/>
@@ -11793,7 +11793,7 @@
       <c r="G242" t="inlineStr"/>
       <c r="H242" t="inlineStr">
         <is>
-          <t>17:03</t>
+          <t>17:02</t>
         </is>
       </c>
       <c r="I242" t="inlineStr"/>
@@ -11840,7 +11840,7 @@
       <c r="G243" t="inlineStr"/>
       <c r="H243" t="inlineStr">
         <is>
-          <t>17:02</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="I243" t="inlineStr"/>
@@ -12780,7 +12780,7 @@
       <c r="G263" t="inlineStr"/>
       <c r="H263" t="inlineStr">
         <is>
-          <t>16:39</t>
+          <t>16:38</t>
         </is>
       </c>
       <c r="I263" t="inlineStr"/>
@@ -13109,7 +13109,7 @@
       <c r="G270" t="inlineStr"/>
       <c r="H270" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:29</t>
         </is>
       </c>
       <c r="I270" t="inlineStr"/>
@@ -13250,7 +13250,7 @@
       <c r="G273" t="inlineStr"/>
       <c r="H273" t="inlineStr">
         <is>
-          <t>16:26</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="I273" t="inlineStr"/>
@@ -13861,7 +13861,7 @@
       <c r="G286" t="inlineStr"/>
       <c r="H286" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>16:08</t>
         </is>
       </c>
       <c r="I286" t="inlineStr"/>
@@ -14190,7 +14190,7 @@
       <c r="G293" t="inlineStr"/>
       <c r="H293" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="I293" t="inlineStr"/>
@@ -14707,7 +14707,7 @@
       <c r="G304" t="inlineStr"/>
       <c r="H304" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:46</t>
         </is>
       </c>
       <c r="I304" t="inlineStr"/>
@@ -14754,7 +14754,7 @@
       <c r="G305" t="inlineStr"/>
       <c r="H305" t="inlineStr">
         <is>
-          <t>15:46</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="I305" t="inlineStr"/>
@@ -15177,7 +15177,7 @@
       <c r="G314" t="inlineStr"/>
       <c r="H314" t="inlineStr">
         <is>
-          <t>14:37</t>
+          <t>14:36</t>
         </is>
       </c>
       <c r="I314" t="inlineStr"/>
@@ -15459,7 +15459,7 @@
       <c r="G320" t="inlineStr"/>
       <c r="H320" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="I320" t="inlineStr"/>
@@ -15600,7 +15600,7 @@
       <c r="G323" t="inlineStr"/>
       <c r="H323" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:29</t>
         </is>
       </c>
       <c r="I323" t="inlineStr"/>
@@ -16070,7 +16070,7 @@
       <c r="G333" t="inlineStr"/>
       <c r="H333" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="I333" t="inlineStr"/>
@@ -16258,7 +16258,7 @@
       <c r="G337" t="inlineStr"/>
       <c r="H337" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:23</t>
         </is>
       </c>
       <c r="I337" t="inlineStr"/>
@@ -16775,7 +16775,7 @@
       <c r="G348" t="inlineStr"/>
       <c r="H348" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:23</t>
         </is>
       </c>
       <c r="I348" t="inlineStr"/>
@@ -17856,7 +17856,7 @@
       <c r="G371" t="inlineStr"/>
       <c r="H371" t="inlineStr">
         <is>
-          <t>14:36</t>
+          <t>14:37</t>
         </is>
       </c>
       <c r="I371" t="inlineStr"/>
@@ -18467,7 +18467,7 @@
       <c r="G384" t="inlineStr"/>
       <c r="H384" t="inlineStr">
         <is>
-          <t>14:49</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="I384" t="inlineStr"/>
@@ -18514,7 +18514,7 @@
       <c r="G385" t="inlineStr"/>
       <c r="H385" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="I385" t="inlineStr"/>
@@ -18890,7 +18890,7 @@
       <c r="G393" t="inlineStr"/>
       <c r="H393" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="I393" t="inlineStr"/>
@@ -18937,7 +18937,7 @@
       <c r="G394" t="inlineStr"/>
       <c r="H394" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="I394" t="inlineStr"/>
@@ -19313,7 +19313,7 @@
       <c r="G402" t="inlineStr"/>
       <c r="H402" t="inlineStr">
         <is>
-          <t>15:09</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="I402" t="inlineStr"/>
@@ -20535,7 +20535,7 @@
       <c r="G428" t="inlineStr"/>
       <c r="H428" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:36</t>
         </is>
       </c>
       <c r="I428" t="inlineStr"/>
@@ -21146,7 +21146,7 @@
       <c r="G441" t="inlineStr"/>
       <c r="H441" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>16:46</t>
         </is>
       </c>
       <c r="I441" t="inlineStr"/>
@@ -21898,7 +21898,7 @@
       <c r="G457" t="inlineStr"/>
       <c r="H457" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="I457" t="inlineStr"/>
@@ -21992,7 +21992,7 @@
       <c r="G459" t="inlineStr"/>
       <c r="H459" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:57</t>
         </is>
       </c>
       <c r="I459" t="inlineStr"/>
@@ -22086,7 +22086,7 @@
       <c r="G461" t="inlineStr"/>
       <c r="H461" t="inlineStr">
         <is>
-          <t>16:57</t>
+          <t>16:58</t>
         </is>
       </c>
       <c r="I461" t="inlineStr"/>
@@ -22180,7 +22180,7 @@
       <c r="G463" t="inlineStr"/>
       <c r="H463" t="inlineStr">
         <is>
-          <t>16:58</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="I463" t="inlineStr"/>
@@ -22274,7 +22274,7 @@
       <c r="G465" t="inlineStr"/>
       <c r="H465" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="I465" t="inlineStr"/>
@@ -22368,7 +22368,7 @@
       <c r="G467" t="inlineStr"/>
       <c r="H467" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="I467" t="inlineStr"/>
@@ -22791,7 +22791,7 @@
       <c r="G476" t="inlineStr"/>
       <c r="H476" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="I476" t="inlineStr"/>
@@ -23026,7 +23026,7 @@
       <c r="G481" t="inlineStr"/>
       <c r="H481" t="inlineStr">
         <is>
-          <t>17:06</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="I481" t="inlineStr"/>
@@ -23261,7 +23261,7 @@
       <c r="G486" t="inlineStr"/>
       <c r="H486" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>17:09</t>
         </is>
       </c>
       <c r="I486" t="inlineStr"/>
@@ -23637,7 +23637,7 @@
       <c r="G494" t="inlineStr"/>
       <c r="H494" t="inlineStr">
         <is>
-          <t>17:11</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="I494" t="inlineStr"/>
@@ -24013,7 +24013,7 @@
       <c r="G502" t="inlineStr"/>
       <c r="H502" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="I502" t="inlineStr"/>
@@ -26927,7 +26927,7 @@
       <c r="G564" t="inlineStr"/>
       <c r="H564" t="inlineStr">
         <is>
-          <t>17:28</t>
+          <t>17:27</t>
         </is>
       </c>
       <c r="I564" t="inlineStr"/>
@@ -27961,7 +27961,7 @@
       <c r="G586" t="inlineStr"/>
       <c r="H586" t="inlineStr">
         <is>
-          <t>17:20</t>
+          <t>17:19</t>
         </is>
       </c>
       <c r="I586" t="inlineStr"/>
@@ -28713,7 +28713,7 @@
       <c r="G602" t="inlineStr"/>
       <c r="H602" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="I602" t="inlineStr"/>
@@ -28760,7 +28760,7 @@
       <c r="G603" t="inlineStr"/>
       <c r="H603" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>17:06</t>
         </is>
       </c>
       <c r="I603" t="inlineStr"/>
@@ -29183,7 +29183,7 @@
       <c r="G612" t="inlineStr"/>
       <c r="H612" t="inlineStr">
         <is>
-          <t>16:58</t>
+          <t>16:57</t>
         </is>
       </c>
       <c r="I612" t="inlineStr"/>
@@ -29230,7 +29230,7 @@
       <c r="G613" t="inlineStr"/>
       <c r="H613" t="inlineStr">
         <is>
-          <t>16:57</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="I613" t="inlineStr"/>
@@ -29559,7 +29559,7 @@
       <c r="G620" t="inlineStr"/>
       <c r="H620" t="inlineStr">
         <is>
-          <t>16:49</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="I620" t="inlineStr"/>
@@ -29794,7 +29794,7 @@
       <c r="G625" t="inlineStr"/>
       <c r="H625" t="inlineStr">
         <is>
-          <t>16:43</t>
+          <t>16:42</t>
         </is>
       </c>
       <c r="I625" t="inlineStr"/>
@@ -29982,7 +29982,7 @@
       <c r="G629" t="inlineStr"/>
       <c r="H629" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:37</t>
         </is>
       </c>
       <c r="I629" t="inlineStr"/>
@@ -30311,7 +30311,7 @@
       <c r="G636" t="inlineStr"/>
       <c r="H636" t="inlineStr">
         <is>
-          <t>16:29</t>
+          <t>16:28</t>
         </is>
       </c>
       <c r="I636" t="inlineStr"/>
@@ -30452,7 +30452,7 @@
       <c r="G639" t="inlineStr"/>
       <c r="H639" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="I639" t="inlineStr"/>
@@ -31063,7 +31063,7 @@
       <c r="G652" t="inlineStr"/>
       <c r="H652" t="inlineStr">
         <is>
-          <t>16:08</t>
+          <t>16:07</t>
         </is>
       </c>
       <c r="I652" t="inlineStr"/>
@@ -31627,7 +31627,7 @@
       <c r="G664" t="inlineStr"/>
       <c r="H664" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:52</t>
         </is>
       </c>
       <c r="I664" t="inlineStr"/>
@@ -32003,7 +32003,7 @@
       <c r="G672" t="inlineStr"/>
       <c r="H672" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="I672" t="inlineStr"/>
@@ -32050,7 +32050,7 @@
       <c r="G673" t="inlineStr"/>
       <c r="H673" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:42</t>
         </is>
       </c>
       <c r="I673" t="inlineStr"/>
@@ -32097,7 +32097,7 @@
       <c r="G674" t="inlineStr"/>
       <c r="H674" t="inlineStr">
         <is>
-          <t>14:42</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="I674" t="inlineStr"/>
@@ -32144,7 +32144,7 @@
       <c r="G675" t="inlineStr"/>
       <c r="H675" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="I675" t="inlineStr"/>
@@ -32191,7 +32191,7 @@
       <c r="G676" t="inlineStr"/>
       <c r="H676" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>14:39</t>
         </is>
       </c>
       <c r="I676" t="inlineStr"/>
@@ -32238,7 +32238,7 @@
       <c r="G677" t="inlineStr"/>
       <c r="H677" t="inlineStr">
         <is>
-          <t>14:39</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="I677" t="inlineStr"/>
@@ -32567,7 +32567,7 @@
       <c r="G684" t="inlineStr"/>
       <c r="H684" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="I684" t="inlineStr"/>
@@ -33413,7 +33413,7 @@
       <c r="G702" t="inlineStr"/>
       <c r="H702" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:23</t>
         </is>
       </c>
       <c r="I702" t="inlineStr"/>
@@ -34118,7 +34118,7 @@
       <c r="G717" t="inlineStr"/>
       <c r="H717" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="I717" t="inlineStr"/>
@@ -34729,7 +34729,7 @@
       <c r="G730" t="inlineStr"/>
       <c r="H730" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="I730" t="inlineStr"/>
@@ -35763,7 +35763,7 @@
       <c r="G752" t="inlineStr"/>
       <c r="H752" t="inlineStr">
         <is>
-          <t>14:52</t>
+          <t>14:53</t>
         </is>
       </c>
       <c r="I752" t="inlineStr"/>
@@ -35810,7 +35810,7 @@
       <c r="G753" t="inlineStr"/>
       <c r="H753" t="inlineStr">
         <is>
-          <t>14:53</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="I753" t="inlineStr"/>
@@ -36186,7 +36186,7 @@
       <c r="G761" t="inlineStr"/>
       <c r="H761" t="inlineStr">
         <is>
-          <t>15:02</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="I761" t="inlineStr"/>
@@ -36562,7 +36562,7 @@
       <c r="G769" t="inlineStr"/>
       <c r="H769" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:12</t>
         </is>
       </c>
       <c r="I769" t="inlineStr"/>
@@ -36609,7 +36609,7 @@
       <c r="G770" t="inlineStr"/>
       <c r="H770" t="inlineStr">
         <is>
-          <t>15:12</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="I770" t="inlineStr"/>
@@ -37596,7 +37596,7 @@
       <c r="G791" t="inlineStr"/>
       <c r="H791" t="inlineStr">
         <is>
-          <t>15:33</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="I791" t="inlineStr"/>
@@ -38113,7 +38113,7 @@
       <c r="G802" t="inlineStr"/>
       <c r="H802" t="inlineStr">
         <is>
-          <t>15:42</t>
+          <t>15:43</t>
         </is>
       </c>
       <c r="I802" t="inlineStr"/>
@@ -38442,7 +38442,7 @@
       <c r="G809" t="inlineStr"/>
       <c r="H809" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="I809" t="inlineStr"/>
@@ -38818,7 +38818,7 @@
       <c r="G817" t="inlineStr"/>
       <c r="H817" t="inlineStr">
         <is>
-          <t>16:52</t>
+          <t>16:53</t>
         </is>
       </c>
       <c r="I817" t="inlineStr"/>
@@ -39852,7 +39852,7 @@
       <c r="G839" t="inlineStr"/>
       <c r="H839" t="inlineStr">
         <is>
-          <t>17:03</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="I839" t="inlineStr"/>
@@ -41309,7 +41309,7 @@
       <c r="G870" t="inlineStr"/>
       <c r="H870" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:16</t>
         </is>
       </c>
       <c r="I870" t="inlineStr"/>
@@ -42437,7 +42437,7 @@
       <c r="G894" t="inlineStr"/>
       <c r="H894" t="inlineStr">
         <is>
-          <t>17:23</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="I894" t="inlineStr"/>
@@ -43001,7 +43001,7 @@
       <c r="G906" t="inlineStr"/>
       <c r="H906" t="inlineStr">
         <is>
-          <t>17:27</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="I906" t="inlineStr"/>
@@ -44505,7 +44505,7 @@
       <c r="G938" t="inlineStr"/>
       <c r="H938" t="inlineStr">
         <is>
-          <t>17:26</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="I938" t="inlineStr"/>
@@ -45539,7 +45539,7 @@
       <c r="G960" t="inlineStr"/>
       <c r="H960" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:13</t>
         </is>
       </c>
       <c r="I960" t="inlineStr"/>
@@ -46479,7 +46479,7 @@
       <c r="G980" t="inlineStr"/>
       <c r="H980" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:54</t>
         </is>
       </c>
       <c r="I980" t="inlineStr"/>
@@ -46808,7 +46808,7 @@
       <c r="G987" t="inlineStr"/>
       <c r="H987" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:46</t>
         </is>
       </c>
       <c r="I987" t="inlineStr"/>
@@ -47184,7 +47184,7 @@
       <c r="G995" t="inlineStr"/>
       <c r="H995" t="inlineStr">
         <is>
-          <t>16:37</t>
+          <t>16:36</t>
         </is>
       </c>
       <c r="I995" t="inlineStr"/>
@@ -47513,7 +47513,7 @@
       <c r="G1002" t="inlineStr"/>
       <c r="H1002" t="inlineStr">
         <is>
-          <t>16:28</t>
+          <t>16:27</t>
         </is>
       </c>
       <c r="I1002" t="inlineStr"/>
@@ -47654,7 +47654,7 @@
       <c r="G1005" t="inlineStr"/>
       <c r="H1005" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="I1005" t="inlineStr"/>
@@ -48265,7 +48265,7 @@
       <c r="G1018" t="inlineStr"/>
       <c r="H1018" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>16:06</t>
         </is>
       </c>
       <c r="I1018" t="inlineStr"/>
@@ -48876,7 +48876,7 @@
       <c r="G1031" t="inlineStr"/>
       <c r="H1031" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="I1031" t="inlineStr"/>
@@ -49675,7 +49675,7 @@
       <c r="G1048" t="inlineStr"/>
       <c r="H1048" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="I1048" t="inlineStr"/>
@@ -49863,7 +49863,7 @@
       <c r="G1052" t="inlineStr"/>
       <c r="H1052" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="I1052" t="inlineStr"/>
@@ -50004,7 +50004,7 @@
       <c r="G1055" t="inlineStr"/>
       <c r="H1055" t="inlineStr">
         <is>
-          <t>14:29</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="I1055" t="inlineStr"/>
@@ -50286,7 +50286,7 @@
       <c r="G1061" t="inlineStr"/>
       <c r="H1061" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="I1061" t="inlineStr"/>

</xml_diff>